<commit_message>
created new exploratory analysis for BERDO AI calculator
</commit_message>
<xml_diff>
--- a/data-files/0-for_narrative/LL84_building_summary_statistics-acp.xlsx
+++ b/data-files/0-for_narrative/LL84_building_summary_statistics-acp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://envienstudio.sharepoint.com/Shared Documents/Potential/DOE RD Submission/3 - Market Research/doe-SBIR-research-project/data-files/0-for_narrative/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="48" documentId="11_DF7ECDD54F75B9BF7F344F9885BE0011C693192A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7FDCEAC2-37F2-46A3-8DEB-5210FAA72493}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="11_DF7ECDD54F75B9BF7F344F9885BE0011C693192A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE63C242-66C3-408C-B22C-55B431D10B33}"/>
   <bookViews>
-    <workbookView xWindow="-14580" yWindow="60" windowWidth="14685" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary with Graphs" sheetId="1" r:id="rId1"/>
@@ -387,8 +387,8 @@
   <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -512,12 +512,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="44" fontId="0" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
@@ -883,6 +883,7 @@
     <col min="12" max="14" width="20.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="12" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="6" customWidth="1"/>
+    <col min="17" max="18" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="20" max="21" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -11467,14 +11468,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d4fe9914-c092-4200-a7d8-cc85a6bef288">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="afc29c3b-9522-4360-ba9d-c1dc5ac90a19" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11727,21 +11726,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d4fe9914-c092-4200-a7d8-cc85a6bef288">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="afc29c3b-9522-4360-ba9d-c1dc5ac90a19" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2903E71-C9DB-4A68-8A9A-DA2967E40696}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA51343D-8703-4BD3-94A2-0CA851CFBDF9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d4fe9914-c092-4200-a7d8-cc85a6bef288"/>
-    <ds:schemaRef ds:uri="afc29c3b-9522-4360-ba9d-c1dc5ac90a19"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11766,9 +11764,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA51343D-8703-4BD3-94A2-0CA851CFBDF9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2903E71-C9DB-4A68-8A9A-DA2967E40696}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d4fe9914-c092-4200-a7d8-cc85a6bef288"/>
+    <ds:schemaRef ds:uri="afc29c3b-9522-4360-ba9d-c1dc5ac90a19"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>